<commit_message>
Added 2 test points
for possible logic level converters
</commit_message>
<xml_diff>
--- a/Release Packages/REV A0 - First Release/Digikey Parts.xlsx
+++ b/Release Packages/REV A0 - First Release/Digikey Parts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d5d13c61c60eae0c/Documents/Space center/Simulation-Main-Board/BOM and Pick and Place Files/REV X4/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d5d13c61c60eae0c/Documents/Space center/Simulation-Main-Board/Release Packages/REV A0 - First Release/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="62" documentId="11_F25DC773A252ABDACC10480A81D964B85ADE58E5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{053CEEFD-359B-4B8E-A64C-B9114D3B9A09}"/>
+  <xr:revisionPtr revIDLastSave="65" documentId="11_F25DC773A252ABDACC10480A81D964B85ADE58E5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53F49BAB-82C0-4930-ADB4-0BACA0148F3D}"/>
   <bookViews>
-    <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10020" yWindow="1416" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -84,28 +84,28 @@
     <t>2223-TS02-66-60-BK-160-LCR-D-ND</t>
   </si>
   <si>
-    <t>455-B9B-EH-A-ND</t>
-  </si>
-  <si>
     <t>J97,J98</t>
   </si>
   <si>
     <t>J13-25, J29-44</t>
   </si>
   <si>
-    <t>455-S3B-PH-KL-ND, or 455-B2B-PH-KL-ND</t>
-  </si>
-  <si>
     <t>J5,J6,J7,J8,J9,J10,J11,J12</t>
   </si>
   <si>
     <t>S9170-ND</t>
   </si>
   <si>
-    <t>455-B4B-EH-A-ND</t>
-  </si>
-  <si>
     <t>J2,J3,J4,J85,J86,J87,J93,J94,J96</t>
+  </si>
+  <si>
+    <t>455-B9B-XH-A-ND</t>
+  </si>
+  <si>
+    <t>455-2248-ND, or 455-B2B-XH-A-ND</t>
+  </si>
+  <si>
+    <t>455-B4B-XH-A-ND</t>
   </si>
 </sst>
 </file>
@@ -431,14 +431,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.21875" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -460,7 +460,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -471,7 +471,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -482,7 +482,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -493,7 +493,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -504,7 +504,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -515,7 +515,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -526,7 +526,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -537,45 +537,45 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C10" s="1">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C11" s="1">
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C12" s="1">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" t="s">
         <v>26</v>
-      </c>
-      <c r="B13" t="s">
-        <v>25</v>
       </c>
       <c r="C13" s="1">
         <v>10</v>

</xml_diff>